<commit_message>
Separate a paper-account reset from a real expiry
Wednesday night's write-offs of CRM, NU and NVDA were not expiries. The
account holder reset the paper account and those positions vanished. IBKR
records a reset exactly as it records an expiry - a sell at price 0 against
lots that were genuinely open - and carries no field that separates the two,
so the distinction cannot be derived; it has to be named. --drop-expiry does
that, and the rows come off on their own audit line.

The week is +$22,486 over 104 exits. The two real expiries stay: MSTR and
PURR on Friday night, 160 contracts, $4,660. Wednesday goes back to -$5,522
and stops breaching rule 15; only Tuesday still does.

check_rules.py takes --vanished SYM@DATE and burn_slices.py a third argument
in the same form, so all three tools see the same week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GTbb2E9cN7NztreWQePDr3
</commit_message>
<xml_diff>
--- a/data/2026-08-24-week/trades-filtered.xlsx
+++ b/data/2026-08-24-week/trades-filtered.xlsx
@@ -13,7 +13,7 @@
     <sheet name="סינון" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'עסקאות'!$A$1:$O$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'עסקאות'!$A$1:$O$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O113"/>
+  <dimension ref="A1:O110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1523,9 @@
         <f>IF(K17=0,"",J17/K17)</f>
         <v/>
       </c>
-      <c r="N17" s="10" t="n"/>
+      <c r="N17" s="10" t="n">
+        <v>4.6</v>
+      </c>
       <c r="O17" s="11" t="n">
         <v>0.77</v>
       </c>
@@ -1580,7 +1582,9 @@
         <f>IF(K18=0,"",J18/K18)</f>
         <v/>
       </c>
-      <c r="N18" s="4" t="n"/>
+      <c r="N18" s="4" t="n">
+        <v>7.4</v>
+      </c>
       <c r="O18" s="5" t="n">
         <v>0.55</v>
       </c>
@@ -1637,7 +1641,9 @@
         <f>IF(K19=0,"",J19/K19)</f>
         <v/>
       </c>
-      <c r="N19" s="10" t="n"/>
+      <c r="N19" s="10" t="n">
+        <v>7.1</v>
+      </c>
       <c r="O19" s="11" t="n">
         <v>1.97</v>
       </c>
@@ -1694,7 +1700,9 @@
         <f>IF(K20=0,"",J20/K20)</f>
         <v/>
       </c>
-      <c r="N20" s="4" t="n"/>
+      <c r="N20" s="4" t="n">
+        <v>7</v>
+      </c>
       <c r="O20" s="5" t="n">
         <v>2.93</v>
       </c>
@@ -1810,7 +1818,9 @@
         <f>IF(K22=0,"",J22/K22)</f>
         <v/>
       </c>
-      <c r="N22" s="4" t="n"/>
+      <c r="N22" s="4" t="n">
+        <v>4.5</v>
+      </c>
       <c r="O22" s="5" t="n">
         <v>6.79</v>
       </c>
@@ -1867,7 +1877,9 @@
         <f>IF(K23=0,"",J23/K23)</f>
         <v/>
       </c>
-      <c r="N23" s="10" t="n"/>
+      <c r="N23" s="10" t="n">
+        <v>13.4</v>
+      </c>
       <c r="O23" s="11" t="n">
         <v>5.43</v>
       </c>
@@ -1983,7 +1995,9 @@
         <f>IF(K25=0,"",J25/K25)</f>
         <v/>
       </c>
-      <c r="N25" s="10" t="n"/>
+      <c r="N25" s="10" t="n">
+        <v>30.6</v>
+      </c>
       <c r="O25" s="11" t="n">
         <v>4.9</v>
       </c>
@@ -2099,7 +2113,9 @@
         <f>IF(K27=0,"",J27/K27)</f>
         <v/>
       </c>
-      <c r="N27" s="10" t="n"/>
+      <c r="N27" s="10" t="n">
+        <v>1.6</v>
+      </c>
       <c r="O27" s="11" t="n">
         <v>4.9</v>
       </c>
@@ -2274,7 +2290,9 @@
         <f>IF(K30=0,"",J30/K30)</f>
         <v/>
       </c>
-      <c r="N30" s="4" t="n"/>
+      <c r="N30" s="4" t="n">
+        <v>13.9</v>
+      </c>
       <c r="O30" s="5" t="n">
         <v>0.79</v>
       </c>
@@ -2331,7 +2349,9 @@
         <f>IF(K31=0,"",J31/K31)</f>
         <v/>
       </c>
-      <c r="N31" s="10" t="n"/>
+      <c r="N31" s="10" t="n">
+        <v>14.7</v>
+      </c>
       <c r="O31" s="11" t="n">
         <v>0.35</v>
       </c>
@@ -2388,7 +2408,9 @@
         <f>IF(K32=0,"",J32/K32)</f>
         <v/>
       </c>
-      <c r="N32" s="4" t="n"/>
+      <c r="N32" s="4" t="n">
+        <v>14.7</v>
+      </c>
       <c r="O32" s="5" t="n">
         <v>8.17</v>
       </c>
@@ -2977,7 +2999,7 @@
         <v/>
       </c>
       <c r="N42" s="4" t="n">
-        <v>72.8</v>
+        <v>118.9</v>
       </c>
       <c r="O42" s="5" t="n">
         <v>6.38</v>
@@ -3811,16 +3833,16 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>רביעי</t>
+          <t>חמישי</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>22:25</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -3834,20 +3856,20 @@
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="G57" s="11" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="H57" s="10">
         <f>IF(F57*G57=0,"",ROUND(I57/(F57*G57),0))</f>
         <v/>
       </c>
       <c r="I57" s="12" t="n">
-        <v>0</v>
+        <v>2760</v>
       </c>
       <c r="J57" s="12" t="n">
-        <v>-1680</v>
+        <v>2358.31</v>
       </c>
       <c r="K57" s="12">
         <f>I57-J57</f>
@@ -3862,29 +3884,29 @@
         <v/>
       </c>
       <c r="N57" s="10" t="n">
-        <v>3305.1</v>
+        <v>1204.6</v>
       </c>
       <c r="O57" s="11" t="n">
-        <v>0</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>רביעי</t>
+          <t>חמישי</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>22:25</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>NU</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
@@ -3893,20 +3915,20 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>340</v>
+        <v>50</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="H58" s="4">
         <f>IF(F58*G58=0,"",ROUND(I58/(F58*G58),0))</f>
         <v/>
       </c>
       <c r="I58" s="6" t="n">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="J58" s="6" t="n">
-        <v>-2940</v>
+        <v>-1166.64</v>
       </c>
       <c r="K58" s="6">
         <f>I58-J58</f>
@@ -3921,29 +3943,29 @@
         <v/>
       </c>
       <c r="N58" s="4" t="n">
-        <v>1883.8</v>
+        <v>2.7</v>
       </c>
       <c r="O58" s="5" t="n">
-        <v>0</v>
+        <v>9.279999999999999</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>רביעי</t>
+          <t>חמישי</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>22:25</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
@@ -3952,20 +3974,20 @@
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="G59" s="11" t="n">
-        <v>0</v>
+        <v>10.45</v>
       </c>
       <c r="H59" s="10">
         <f>IF(F59*G59=0,"",ROUND(I59/(F59*G59),0))</f>
         <v/>
       </c>
       <c r="I59" s="12" t="n">
-        <v>0</v>
+        <v>4180</v>
       </c>
       <c r="J59" s="12" t="n">
-        <v>-1891</v>
+        <v>3778.28</v>
       </c>
       <c r="K59" s="12">
         <f>I59-J59</f>
@@ -3980,10 +4002,10 @@
         <v/>
       </c>
       <c r="N59" s="10" t="n">
-        <v>584.8</v>
+        <v>1211</v>
       </c>
       <c r="O59" s="11" t="n">
-        <v>0</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="60">
@@ -3997,7 +4019,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -4011,20 +4033,20 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>6.9</v>
+        <v>3.7</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60*G60=0,"",ROUND(I60/(F60*G60),0))</f>
         <v/>
       </c>
       <c r="I60" s="6" t="n">
-        <v>2760</v>
+        <v>5550</v>
       </c>
       <c r="J60" s="6" t="n">
-        <v>2358.31</v>
+        <v>5194.55</v>
       </c>
       <c r="K60" s="6">
         <f>I60-J60</f>
@@ -4039,10 +4061,10 @@
         <v/>
       </c>
       <c r="N60" s="4" t="n">
-        <v>1204.6</v>
+        <v>1215.3</v>
       </c>
       <c r="O60" s="5" t="n">
-        <v>1.14</v>
+        <v>4.47</v>
       </c>
     </row>
     <row r="61">
@@ -4056,12 +4078,12 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>09:36</t>
+          <t>09:47</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
@@ -4070,20 +4092,20 @@
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G61" s="11" t="n">
-        <v>0.19</v>
+        <v>2.81</v>
       </c>
       <c r="H61" s="10">
         <f>IF(F61*G61=0,"",ROUND(I61/(F61*G61),0))</f>
         <v/>
       </c>
       <c r="I61" s="12" t="n">
-        <v>950</v>
+        <v>1405</v>
       </c>
       <c r="J61" s="12" t="n">
-        <v>-1166.64</v>
+        <v>1070.89</v>
       </c>
       <c r="K61" s="12">
         <f>I61-J61</f>
@@ -4098,10 +4120,10 @@
         <v/>
       </c>
       <c r="N61" s="10" t="n">
-        <v>2.7</v>
+        <v>1198.5</v>
       </c>
       <c r="O61" s="11" t="n">
-        <v>9.279999999999999</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="62">
@@ -4115,12 +4137,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:48</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
@@ -4129,20 +4151,20 @@
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>10.45</v>
+        <v>2.34</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62*G62=0,"",ROUND(I62/(F62*G62),0))</f>
         <v/>
       </c>
       <c r="I62" s="6" t="n">
-        <v>4180</v>
+        <v>468</v>
       </c>
       <c r="J62" s="6" t="n">
-        <v>3778.28</v>
+        <v>334.52</v>
       </c>
       <c r="K62" s="6">
         <f>I62-J62</f>
@@ -4157,10 +4179,10 @@
         <v/>
       </c>
       <c r="N62" s="4" t="n">
-        <v>1211</v>
+        <v>1199.1</v>
       </c>
       <c r="O62" s="5" t="n">
-        <v>1.17</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="63">
@@ -4174,12 +4196,12 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
@@ -4188,20 +4210,20 @@
         </is>
       </c>
       <c r="F63" s="10" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="G63" s="11" t="n">
-        <v>3.7</v>
+        <v>0.2</v>
       </c>
       <c r="H63" s="10">
         <f>IF(F63*G63=0,"",ROUND(I63/(F63*G63),0))</f>
         <v/>
       </c>
       <c r="I63" s="12" t="n">
-        <v>5550</v>
+        <v>1100</v>
       </c>
       <c r="J63" s="12" t="n">
-        <v>5194.55</v>
+        <v>-1138.26</v>
       </c>
       <c r="K63" s="12">
         <f>I63-J63</f>
@@ -4216,10 +4238,10 @@
         <v/>
       </c>
       <c r="N63" s="10" t="n">
-        <v>1215.3</v>
+        <v>8.9</v>
       </c>
       <c r="O63" s="11" t="n">
-        <v>4.47</v>
+        <v>26.85</v>
       </c>
     </row>
     <row r="64">
@@ -4233,12 +4255,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>09:47</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
@@ -4247,20 +4269,20 @@
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>2.81</v>
+        <v>3.15</v>
       </c>
       <c r="H64" s="4">
         <f>IF(F64*G64=0,"",ROUND(I64/(F64*G64),0))</f>
         <v/>
       </c>
       <c r="I64" s="6" t="n">
-        <v>1405</v>
+        <v>4725</v>
       </c>
       <c r="J64" s="6" t="n">
-        <v>1070.89</v>
+        <v>4369.94</v>
       </c>
       <c r="K64" s="6">
         <f>I64-J64</f>
@@ -4275,10 +4297,10 @@
         <v/>
       </c>
       <c r="N64" s="4" t="n">
-        <v>1198.5</v>
+        <v>1225.9</v>
       </c>
       <c r="O64" s="5" t="n">
-        <v>1.77</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="65">
@@ -4292,12 +4314,12 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>09:48</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -4306,20 +4328,20 @@
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G65" s="11" t="n">
-        <v>2.34</v>
+        <v>1.4</v>
       </c>
       <c r="H65" s="10">
         <f>IF(F65*G65=0,"",ROUND(I65/(F65*G65),0))</f>
         <v/>
       </c>
       <c r="I65" s="12" t="n">
-        <v>468</v>
+        <v>2800</v>
       </c>
       <c r="J65" s="12" t="n">
-        <v>334.52</v>
+        <v>1524.46</v>
       </c>
       <c r="K65" s="12">
         <f>I65-J65</f>
@@ -4334,10 +4356,10 @@
         <v/>
       </c>
       <c r="N65" s="10" t="n">
-        <v>1199.1</v>
+        <v>18.2</v>
       </c>
       <c r="O65" s="11" t="n">
-        <v>0.55</v>
+        <v>7.48</v>
       </c>
     </row>
     <row r="66">
@@ -4351,12 +4373,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -4365,20 +4387,20 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>0.2</v>
+        <v>4.9</v>
       </c>
       <c r="H66" s="4">
         <f>IF(F66*G66=0,"",ROUND(I66/(F66*G66),0))</f>
         <v/>
       </c>
       <c r="I66" s="6" t="n">
-        <v>1100</v>
+        <v>4900</v>
       </c>
       <c r="J66" s="6" t="n">
-        <v>-1138.26</v>
+        <v>4663.21</v>
       </c>
       <c r="K66" s="6">
         <f>I66-J66</f>
@@ -4393,10 +4415,10 @@
         <v/>
       </c>
       <c r="N66" s="4" t="n">
-        <v>8.9</v>
+        <v>1239.8</v>
       </c>
       <c r="O66" s="5" t="n">
-        <v>26.85</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="67">
@@ -4410,12 +4432,12 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
@@ -4424,20 +4446,20 @@
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G67" s="11" t="n">
-        <v>3.15</v>
+        <v>2.06</v>
       </c>
       <c r="H67" s="10">
         <f>IF(F67*G67=0,"",ROUND(I67/(F67*G67),0))</f>
         <v/>
       </c>
       <c r="I67" s="12" t="n">
-        <v>4725</v>
+        <v>4738</v>
       </c>
       <c r="J67" s="12" t="n">
-        <v>4369.94</v>
+        <v>3207.33</v>
       </c>
       <c r="K67" s="12">
         <f>I67-J67</f>
@@ -4452,10 +4474,10 @@
         <v/>
       </c>
       <c r="N67" s="10" t="n">
-        <v>1225.9</v>
+        <v>1226.3</v>
       </c>
       <c r="O67" s="11" t="n">
-        <v>4.07</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="68">
@@ -4469,12 +4491,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
@@ -4483,20 +4505,20 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>1.4</v>
+        <v>0.26</v>
       </c>
       <c r="H68" s="4">
         <f>IF(F68*G68=0,"",ROUND(I68/(F68*G68),0))</f>
         <v/>
       </c>
       <c r="I68" s="6" t="n">
-        <v>2800</v>
+        <v>1690</v>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1524.46</v>
+        <v>-233.68</v>
       </c>
       <c r="K68" s="6">
         <f>I68-J68</f>
@@ -4511,10 +4533,10 @@
         <v/>
       </c>
       <c r="N68" s="4" t="n">
-        <v>18.2</v>
+        <v>3.8</v>
       </c>
       <c r="O68" s="5" t="n">
-        <v>7.48</v>
+        <v>11.33</v>
       </c>
     </row>
     <row r="69">
@@ -4528,7 +4550,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -4542,20 +4564,20 @@
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G69" s="11" t="n">
-        <v>4.9</v>
+        <v>6.8</v>
       </c>
       <c r="H69" s="10">
         <f>IF(F69*G69=0,"",ROUND(I69/(F69*G69),0))</f>
         <v/>
       </c>
       <c r="I69" s="12" t="n">
-        <v>4900</v>
+        <v>1360</v>
       </c>
       <c r="J69" s="12" t="n">
-        <v>4663.21</v>
+        <v>1312.59</v>
       </c>
       <c r="K69" s="12">
         <f>I69-J69</f>
@@ -4570,10 +4592,10 @@
         <v/>
       </c>
       <c r="N69" s="10" t="n">
-        <v>1239.8</v>
+        <v>1254.6</v>
       </c>
       <c r="O69" s="11" t="n">
-        <v>2.81</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="70">
@@ -4587,12 +4609,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -4601,20 +4623,20 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>2.06</v>
+        <v>6.9</v>
       </c>
       <c r="H70" s="4">
         <f>IF(F70*G70=0,"",ROUND(I70/(F70*G70),0))</f>
         <v/>
       </c>
       <c r="I70" s="6" t="n">
-        <v>4738</v>
+        <v>2760</v>
       </c>
       <c r="J70" s="6" t="n">
-        <v>3207.33</v>
+        <v>2665.21</v>
       </c>
       <c r="K70" s="6">
         <f>I70-J70</f>
@@ -4629,10 +4651,10 @@
         <v/>
       </c>
       <c r="N70" s="4" t="n">
-        <v>1226.3</v>
+        <v>1142.7</v>
       </c>
       <c r="O70" s="5" t="n">
-        <v>1.93</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="71">
@@ -4646,12 +4668,12 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
@@ -4660,20 +4682,20 @@
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="G71" s="11" t="n">
-        <v>0.26</v>
+        <v>6.8</v>
       </c>
       <c r="H71" s="10">
         <f>IF(F71*G71=0,"",ROUND(I71/(F71*G71),0))</f>
         <v/>
       </c>
       <c r="I71" s="12" t="n">
-        <v>1690</v>
+        <v>9520</v>
       </c>
       <c r="J71" s="12" t="n">
-        <v>-233.68</v>
+        <v>9188.15</v>
       </c>
       <c r="K71" s="12">
         <f>I71-J71</f>
@@ -4688,10 +4710,10 @@
         <v/>
       </c>
       <c r="N71" s="10" t="n">
-        <v>3.8</v>
+        <v>1222.8</v>
       </c>
       <c r="O71" s="11" t="n">
-        <v>11.33</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="72">
@@ -4705,12 +4727,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:39</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -4719,20 +4741,20 @@
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>6.8</v>
+        <v>0.06</v>
       </c>
       <c r="H72" s="4">
         <f>IF(F72*G72=0,"",ROUND(I72/(F72*G72),0))</f>
         <v/>
       </c>
       <c r="I72" s="6" t="n">
-        <v>1360</v>
+        <v>750</v>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1312.59</v>
+        <v>-972.03</v>
       </c>
       <c r="K72" s="6">
         <f>I72-J72</f>
@@ -4747,10 +4769,10 @@
         <v/>
       </c>
       <c r="N72" s="4" t="n">
-        <v>1254.6</v>
+        <v>14.3</v>
       </c>
       <c r="O72" s="5" t="n">
-        <v>0.61</v>
+        <v>32.26</v>
       </c>
     </row>
     <row r="73">
@@ -4764,12 +4786,12 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:39</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
@@ -4778,20 +4800,20 @@
         </is>
       </c>
       <c r="F73" s="10" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="G73" s="11" t="n">
-        <v>6.9</v>
+        <v>0.27</v>
       </c>
       <c r="H73" s="10">
         <f>IF(F73*G73=0,"",ROUND(I73/(F73*G73),0))</f>
         <v/>
       </c>
       <c r="I73" s="12" t="n">
-        <v>2760</v>
+        <v>2160</v>
       </c>
       <c r="J73" s="12" t="n">
-        <v>2665.21</v>
+        <v>-1567.09</v>
       </c>
       <c r="K73" s="12">
         <f>I73-J73</f>
@@ -4806,10 +4828,10 @@
         <v/>
       </c>
       <c r="N73" s="10" t="n">
-        <v>1142.7</v>
+        <v>51.1</v>
       </c>
       <c r="O73" s="11" t="n">
-        <v>1.19</v>
+        <v>22.25</v>
       </c>
     </row>
     <row r="74">
@@ -4823,12 +4845,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
@@ -4837,20 +4859,20 @@
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>6.8</v>
+        <v>1.08</v>
       </c>
       <c r="H74" s="4">
         <f>IF(F74*G74=0,"",ROUND(I74/(F74*G74),0))</f>
         <v/>
       </c>
       <c r="I74" s="6" t="n">
-        <v>9520</v>
+        <v>2700</v>
       </c>
       <c r="J74" s="6" t="n">
-        <v>9188.15</v>
+        <v>1108.1</v>
       </c>
       <c r="K74" s="6">
         <f>I74-J74</f>
@@ -4865,10 +4887,10 @@
         <v/>
       </c>
       <c r="N74" s="4" t="n">
-        <v>1222.8</v>
+        <v>45.6</v>
       </c>
       <c r="O74" s="5" t="n">
-        <v>4.26</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="75">
@@ -4882,12 +4904,12 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>10:39</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
@@ -4896,20 +4918,20 @@
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>125</v>
+        <v>40</v>
       </c>
       <c r="G75" s="11" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="H75" s="10">
         <f>IF(F75*G75=0,"",ROUND(I75/(F75*G75),0))</f>
         <v/>
       </c>
       <c r="I75" s="12" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="J75" s="12" t="n">
-        <v>-972.03</v>
+        <v>-1021.54</v>
       </c>
       <c r="K75" s="12">
         <f>I75-J75</f>
@@ -4924,10 +4946,10 @@
         <v/>
       </c>
       <c r="N75" s="10" t="n">
-        <v>14.3</v>
+        <v>69.2</v>
       </c>
       <c r="O75" s="11" t="n">
-        <v>32.26</v>
+        <v>10.84</v>
       </c>
     </row>
     <row r="76">
@@ -4941,12 +4963,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>10:39</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -4955,20 +4977,20 @@
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>0.27</v>
+        <v>2.5</v>
       </c>
       <c r="H76" s="4">
         <f>IF(F76*G76=0,"",ROUND(I76/(F76*G76),0))</f>
         <v/>
       </c>
       <c r="I76" s="6" t="n">
-        <v>2160</v>
+        <v>8750</v>
       </c>
       <c r="J76" s="6" t="n">
-        <v>-1567.09</v>
+        <v>3879.51</v>
       </c>
       <c r="K76" s="6">
         <f>I76-J76</f>
@@ -4983,10 +5005,10 @@
         <v/>
       </c>
       <c r="N76" s="4" t="n">
-        <v>51.1</v>
+        <v>106.2</v>
       </c>
       <c r="O76" s="5" t="n">
-        <v>22.25</v>
+        <v>9.43</v>
       </c>
     </row>
     <row r="77">
@@ -5000,12 +5022,12 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
@@ -5014,20 +5036,20 @@
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="G77" s="11" t="n">
-        <v>1.08</v>
+        <v>0.18</v>
       </c>
       <c r="H77" s="10">
         <f>IF(F77*G77=0,"",ROUND(I77/(F77*G77),0))</f>
         <v/>
       </c>
       <c r="I77" s="12" t="n">
-        <v>2700</v>
+        <v>1440</v>
       </c>
       <c r="J77" s="12" t="n">
-        <v>1108.1</v>
+        <v>-843.71</v>
       </c>
       <c r="K77" s="12">
         <f>I77-J77</f>
@@ -5042,10 +5064,10 @@
         <v/>
       </c>
       <c r="N77" s="10" t="n">
-        <v>45.6</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="O77" s="11" t="n">
-        <v>6.82</v>
+        <v>22.32</v>
       </c>
     </row>
     <row r="78">
@@ -5059,34 +5081,34 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>13:06</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>FOP</t>
         </is>
       </c>
       <c r="F78" s="4" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>0.25</v>
+        <v>0.85</v>
       </c>
       <c r="H78" s="4">
         <f>IF(F78*G78=0,"",ROUND(I78/(F78*G78),0))</f>
         <v/>
       </c>
       <c r="I78" s="6" t="n">
-        <v>1000</v>
+        <v>1147.5</v>
       </c>
       <c r="J78" s="6" t="n">
-        <v>-1021.54</v>
+        <v>-413.64</v>
       </c>
       <c r="K78" s="6">
         <f>I78-J78</f>
@@ -5101,10 +5123,10 @@
         <v/>
       </c>
       <c r="N78" s="4" t="n">
-        <v>69.2</v>
+        <v>25.8</v>
       </c>
       <c r="O78" s="5" t="n">
-        <v>10.84</v>
+        <v>38.07</v>
       </c>
     </row>
     <row r="79">
@@ -5118,34 +5140,34 @@
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>FOP</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="G79" s="11" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="H79" s="10">
         <f>IF(F79*G79=0,"",ROUND(I79/(F79*G79),0))</f>
         <v/>
       </c>
       <c r="I79" s="12" t="n">
-        <v>8750</v>
+        <v>120</v>
       </c>
       <c r="J79" s="12" t="n">
-        <v>3879.51</v>
+        <v>-53.46</v>
       </c>
       <c r="K79" s="12">
         <f>I79-J79</f>
@@ -5160,10 +5182,10 @@
         <v/>
       </c>
       <c r="N79" s="10" t="n">
-        <v>106.2</v>
+        <v>26.3</v>
       </c>
       <c r="O79" s="11" t="n">
-        <v>9.43</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="80">
@@ -5177,12 +5199,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>11:37</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -5191,20 +5213,20 @@
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>0.18</v>
+        <v>0.49</v>
       </c>
       <c r="H80" s="4">
         <f>IF(F80*G80=0,"",ROUND(I80/(F80*G80),0))</f>
         <v/>
       </c>
       <c r="I80" s="6" t="n">
-        <v>1440</v>
+        <v>1960</v>
       </c>
       <c r="J80" s="6" t="n">
-        <v>-843.71</v>
+        <v>-532.62</v>
       </c>
       <c r="K80" s="6">
         <f>I80-J80</f>
@@ -5219,10 +5241,10 @@
         <v/>
       </c>
       <c r="N80" s="4" t="n">
-        <v>66.90000000000001</v>
+        <v>54.9</v>
       </c>
       <c r="O80" s="5" t="n">
-        <v>22.32</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="81">
@@ -5236,34 +5258,34 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>13:06</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>FOP</t>
+          <t>FUT</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G81" s="11" t="n">
-        <v>0.85</v>
+        <v>84.18000000000001</v>
       </c>
       <c r="H81" s="10">
         <f>IF(F81*G81=0,"",ROUND(I81/(F81*G81),0))</f>
         <v/>
       </c>
       <c r="I81" s="12" t="n">
-        <v>1147.5</v>
+        <v>168360</v>
       </c>
       <c r="J81" s="12" t="n">
-        <v>-413.64</v>
+        <v>1210.56</v>
       </c>
       <c r="K81" s="12">
         <f>I81-J81</f>
@@ -5278,10 +5300,10 @@
         <v/>
       </c>
       <c r="N81" s="10" t="n">
-        <v>25.8</v>
+        <v>7.4</v>
       </c>
       <c r="O81" s="11" t="n">
-        <v>38.07</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="82">
@@ -5295,34 +5317,34 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>FOP</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="F82" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H82" s="4">
         <f>IF(F82*G82=0,"",ROUND(I82/(F82*G82),0))</f>
         <v/>
       </c>
       <c r="I82" s="6" t="n">
-        <v>120</v>
+        <v>770</v>
       </c>
       <c r="J82" s="6" t="n">
-        <v>-53.46</v>
+        <v>284.42</v>
       </c>
       <c r="K82" s="6">
         <f>I82-J82</f>
@@ -5337,10 +5359,10 @@
         <v/>
       </c>
       <c r="N82" s="4" t="n">
-        <v>26.3</v>
+        <v>104.7</v>
       </c>
       <c r="O82" s="5" t="n">
-        <v>4.23</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="83">
@@ -5354,12 +5376,12 @@
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
@@ -5368,20 +5390,20 @@
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="G83" s="11" t="n">
-        <v>0.49</v>
+        <v>0.71</v>
       </c>
       <c r="H83" s="10">
         <f>IF(F83*G83=0,"",ROUND(I83/(F83*G83),0))</f>
         <v/>
       </c>
       <c r="I83" s="12" t="n">
-        <v>1960</v>
+        <v>284</v>
       </c>
       <c r="J83" s="12" t="n">
-        <v>-532.62</v>
+        <v>107.52</v>
       </c>
       <c r="K83" s="12">
         <f>I83-J83</f>
@@ -5396,10 +5418,10 @@
         <v/>
       </c>
       <c r="N83" s="10" t="n">
-        <v>54.9</v>
+        <v>104.6</v>
       </c>
       <c r="O83" s="11" t="n">
-        <v>4.95</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="84">
@@ -5413,7 +5435,7 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -5427,20 +5449,20 @@
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>84.18000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="H84" s="4">
         <f>IF(F84*G84=0,"",ROUND(I84/(F84*G84),0))</f>
         <v/>
       </c>
       <c r="I84" s="6" t="n">
-        <v>168360</v>
+        <v>250410</v>
       </c>
       <c r="J84" s="6" t="n">
-        <v>1210.56</v>
+        <v>-314.16</v>
       </c>
       <c r="K84" s="6">
         <f>I84-J84</f>
@@ -5455,10 +5477,10 @@
         <v/>
       </c>
       <c r="N84" s="4" t="n">
-        <v>7.4</v>
+        <v>33.2</v>
       </c>
       <c r="O84" s="5" t="n">
-        <v>4.72</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="85">
@@ -5472,12 +5494,12 @@
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -5486,20 +5508,20 @@
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="G85" s="11" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="H85" s="10">
         <f>IF(F85*G85=0,"",ROUND(I85/(F85*G85),0))</f>
         <v/>
       </c>
       <c r="I85" s="12" t="n">
-        <v>770</v>
+        <v>1000</v>
       </c>
       <c r="J85" s="12" t="n">
-        <v>284.42</v>
+        <v>-1462.93</v>
       </c>
       <c r="K85" s="12">
         <f>I85-J85</f>
@@ -5514,10 +5536,10 @@
         <v/>
       </c>
       <c r="N85" s="10" t="n">
-        <v>104.7</v>
+        <v>225.8</v>
       </c>
       <c r="O85" s="11" t="n">
-        <v>3.39</v>
+        <v>29.52</v>
       </c>
     </row>
     <row r="86">
@@ -5531,7 +5553,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -5545,20 +5567,20 @@
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>0.71</v>
+        <v>0.97</v>
       </c>
       <c r="H86" s="4">
         <f>IF(F86*G86=0,"",ROUND(I86/(F86*G86),0))</f>
         <v/>
       </c>
       <c r="I86" s="6" t="n">
-        <v>284</v>
+        <v>194</v>
       </c>
       <c r="J86" s="6" t="n">
-        <v>107.52</v>
+        <v>105.79</v>
       </c>
       <c r="K86" s="6">
         <f>I86-J86</f>
@@ -5573,10 +5595,10 @@
         <v/>
       </c>
       <c r="N86" s="4" t="n">
-        <v>104.6</v>
+        <v>217.3</v>
       </c>
       <c r="O86" s="5" t="n">
-        <v>1.14</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="87">
@@ -5590,34 +5612,34 @@
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>FUT</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="G87" s="11" t="n">
-        <v>83.47</v>
+        <v>0.99</v>
       </c>
       <c r="H87" s="10">
         <f>IF(F87*G87=0,"",ROUND(I87/(F87*G87),0))</f>
         <v/>
       </c>
       <c r="I87" s="12" t="n">
-        <v>250410</v>
+        <v>2178</v>
       </c>
       <c r="J87" s="12" t="n">
-        <v>-314.16</v>
+        <v>1204.76</v>
       </c>
       <c r="K87" s="12">
         <f>I87-J87</f>
@@ -5632,10 +5654,10 @@
         <v/>
       </c>
       <c r="N87" s="10" t="n">
-        <v>33.2</v>
+        <v>216.9</v>
       </c>
       <c r="O87" s="11" t="n">
-        <v>7.08</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -5649,12 +5671,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
@@ -5663,20 +5685,20 @@
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>0.1</v>
+        <v>0.97</v>
       </c>
       <c r="H88" s="4">
         <f>IF(F88*G88=0,"",ROUND(I88/(F88*G88),0))</f>
         <v/>
       </c>
       <c r="I88" s="6" t="n">
-        <v>1000</v>
+        <v>97</v>
       </c>
       <c r="J88" s="6" t="n">
-        <v>-1462.93</v>
+        <v>52.89</v>
       </c>
       <c r="K88" s="6">
         <f>I88-J88</f>
@@ -5691,10 +5713,10 @@
         <v/>
       </c>
       <c r="N88" s="4" t="n">
-        <v>225.8</v>
+        <v>217.7</v>
       </c>
       <c r="O88" s="5" t="n">
-        <v>29.52</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="89">
@@ -5708,34 +5730,34 @@
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>23:08</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>FOP</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G89" s="11" t="n">
-        <v>0.97</v>
+        <v>0.03</v>
       </c>
       <c r="H89" s="10">
         <f>IF(F89*G89=0,"",ROUND(I89/(F89*G89),0))</f>
         <v/>
       </c>
       <c r="I89" s="12" t="n">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="J89" s="12" t="n">
-        <v>105.79</v>
+        <v>-1433.04</v>
       </c>
       <c r="K89" s="12">
         <f>I89-J89</f>
@@ -5750,10 +5772,10 @@
         <v/>
       </c>
       <c r="N89" s="10" t="n">
-        <v>217.3</v>
+        <v>546.4</v>
       </c>
       <c r="O89" s="11" t="n">
-        <v>0.55</v>
+        <v>16.52</v>
       </c>
     </row>
     <row r="90">
@@ -5767,34 +5789,34 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>23:16</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>FOP</t>
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>0.99</v>
+        <v>0.03</v>
       </c>
       <c r="H90" s="4">
         <f>IF(F90*G90=0,"",ROUND(I90/(F90*G90),0))</f>
         <v/>
       </c>
       <c r="I90" s="6" t="n">
-        <v>2178</v>
+        <v>150</v>
       </c>
       <c r="J90" s="6" t="n">
-        <v>1204.76</v>
+        <v>-1023.6</v>
       </c>
       <c r="K90" s="6">
         <f>I90-J90</f>
@@ -5809,51 +5831,51 @@
         <v/>
       </c>
       <c r="N90" s="4" t="n">
-        <v>216.9</v>
+        <v>555.1</v>
       </c>
       <c r="O90" s="5" t="n">
-        <v>8.869999999999999</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>חמישי</t>
+          <t>שישי</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>FUT</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G91" s="11" t="n">
-        <v>0.97</v>
+        <v>29612.5</v>
       </c>
       <c r="H91" s="10">
         <f>IF(F91*G91=0,"",ROUND(I91/(F91*G91),0))</f>
         <v/>
       </c>
       <c r="I91" s="12" t="n">
-        <v>97</v>
+        <v>592250</v>
       </c>
       <c r="J91" s="12" t="n">
-        <v>52.89</v>
+        <v>0</v>
       </c>
       <c r="K91" s="12">
         <f>I91-J91</f>
@@ -5867,52 +5889,50 @@
         <f>IF(K91=0,"",J91/K91)</f>
         <v/>
       </c>
-      <c r="N91" s="10" t="n">
-        <v>217.7</v>
-      </c>
+      <c r="N91" s="10" t="n"/>
       <c r="O91" s="11" t="n">
-        <v>0.27</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>חמישי</t>
+          <t>שישי</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>23:08</t>
+          <t>09:32</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>FOP</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>0.03</v>
+        <v>0.21</v>
       </c>
       <c r="H92" s="4">
         <f>IF(F92*G92=0,"",ROUND(I92/(F92*G92),0))</f>
         <v/>
       </c>
       <c r="I92" s="6" t="n">
-        <v>210</v>
+        <v>1365</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>-1433.04</v>
+        <v>-814.5599999999999</v>
       </c>
       <c r="K92" s="6">
         <f>I92-J92</f>
@@ -5927,51 +5947,51 @@
         <v/>
       </c>
       <c r="N92" s="4" t="n">
-        <v>546.4</v>
+        <v>0.6</v>
       </c>
       <c r="O92" s="5" t="n">
-        <v>16.52</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>חמישי</t>
+          <t>שישי</t>
         </is>
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>23:16</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>FOP</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="G93" s="11" t="n">
-        <v>0.03</v>
+        <v>0.16</v>
       </c>
       <c r="H93" s="10">
         <f>IF(F93*G93=0,"",ROUND(I93/(F93*G93),0))</f>
         <v/>
       </c>
       <c r="I93" s="12" t="n">
-        <v>150</v>
+        <v>1120</v>
       </c>
       <c r="J93" s="12" t="n">
-        <v>-1023.6</v>
+        <v>-1233.84</v>
       </c>
       <c r="K93" s="12">
         <f>I93-J93</f>
@@ -5986,10 +6006,10 @@
         <v/>
       </c>
       <c r="N93" s="10" t="n">
-        <v>555.1</v>
+        <v>7</v>
       </c>
       <c r="O93" s="11" t="n">
-        <v>11.8</v>
+        <v>18.96</v>
       </c>
     </row>
     <row r="94">
@@ -6003,34 +6023,34 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>01:23</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>FUT</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="F94" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G94" s="5" t="n">
-        <v>29612.5</v>
+        <v>2.34</v>
       </c>
       <c r="H94" s="4">
         <f>IF(F94*G94=0,"",ROUND(I94/(F94*G94),0))</f>
         <v/>
       </c>
       <c r="I94" s="6" t="n">
-        <v>592250</v>
+        <v>2340</v>
       </c>
       <c r="J94" s="6" t="n">
-        <v>0</v>
+        <v>1892.49</v>
       </c>
       <c r="K94" s="6">
         <f>I94-J94</f>
@@ -6044,9 +6064,11 @@
         <f>IF(K94=0,"",J94/K94)</f>
         <v/>
       </c>
-      <c r="N94" s="4" t="n"/>
+      <c r="N94" s="4" t="n">
+        <v>1287</v>
+      </c>
       <c r="O94" s="5" t="n">
-        <v>2.24</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="95">
@@ -6060,12 +6082,12 @@
       </c>
       <c r="C95" s="9" t="inlineStr">
         <is>
-          <t>09:32</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
@@ -6074,20 +6096,20 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G95" s="11" t="n">
-        <v>0.21</v>
+        <v>0.05</v>
       </c>
       <c r="H95" s="10">
         <f>IF(F95*G95=0,"",ROUND(I95/(F95*G95),0))</f>
         <v/>
       </c>
       <c r="I95" s="12" t="n">
-        <v>1365</v>
+        <v>350</v>
       </c>
       <c r="J95" s="12" t="n">
-        <v>-814.5599999999999</v>
+        <v>-2070.79</v>
       </c>
       <c r="K95" s="12">
         <f>I95-J95</f>
@@ -6102,10 +6124,10 @@
         <v/>
       </c>
       <c r="N95" s="10" t="n">
-        <v>0.6</v>
+        <v>1078.9</v>
       </c>
       <c r="O95" s="11" t="n">
-        <v>26.8</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="96">
@@ -6119,12 +6141,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
@@ -6133,7 +6155,7 @@
         </is>
       </c>
       <c r="F96" s="4" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="G96" s="5" t="n">
         <v>0.16</v>
@@ -6143,10 +6165,10 @@
         <v/>
       </c>
       <c r="I96" s="6" t="n">
-        <v>1120</v>
+        <v>16</v>
       </c>
       <c r="J96" s="6" t="n">
-        <v>-1233.84</v>
+        <v>-56.8</v>
       </c>
       <c r="K96" s="6">
         <f>I96-J96</f>
@@ -6161,10 +6183,10 @@
         <v/>
       </c>
       <c r="N96" s="4" t="n">
-        <v>7</v>
+        <v>1077.1</v>
       </c>
       <c r="O96" s="5" t="n">
-        <v>18.96</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="97">
@@ -6178,12 +6200,12 @@
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
@@ -6192,20 +6214,20 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="G97" s="11" t="n">
-        <v>2.34</v>
+        <v>0.14</v>
       </c>
       <c r="H97" s="10">
         <f>IF(F97*G97=0,"",ROUND(I97/(F97*G97),0))</f>
         <v/>
       </c>
       <c r="I97" s="12" t="n">
-        <v>2340</v>
+        <v>406</v>
       </c>
       <c r="J97" s="12" t="n">
-        <v>1892.49</v>
+        <v>-1689.42</v>
       </c>
       <c r="K97" s="12">
         <f>I97-J97</f>
@@ -6220,10 +6242,10 @@
         <v/>
       </c>
       <c r="N97" s="10" t="n">
-        <v>1287</v>
+        <v>1077.6</v>
       </c>
       <c r="O97" s="11" t="n">
-        <v>4.15</v>
+        <v>7.23</v>
       </c>
     </row>
     <row r="98">
@@ -6237,12 +6259,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
@@ -6251,20 +6273,20 @@
         </is>
       </c>
       <c r="F98" s="4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G98" s="5" t="n">
-        <v>0.05</v>
+        <v>0.18</v>
       </c>
       <c r="H98" s="4">
         <f>IF(F98*G98=0,"",ROUND(I98/(F98*G98),0))</f>
         <v/>
       </c>
       <c r="I98" s="6" t="n">
-        <v>350</v>
+        <v>1080</v>
       </c>
       <c r="J98" s="6" t="n">
-        <v>-2070.79</v>
+        <v>-568.15</v>
       </c>
       <c r="K98" s="6">
         <f>I98-J98</f>
@@ -6279,10 +6301,10 @@
         <v/>
       </c>
       <c r="N98" s="4" t="n">
-        <v>1078.9</v>
+        <v>10.4</v>
       </c>
       <c r="O98" s="5" t="n">
-        <v>36.7</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="99">
@@ -6296,12 +6318,12 @@
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
@@ -6310,20 +6332,20 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="G99" s="11" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="H99" s="10">
         <f>IF(F99*G99=0,"",ROUND(I99/(F99*G99),0))</f>
         <v/>
       </c>
       <c r="I99" s="12" t="n">
-        <v>16</v>
+        <v>1062</v>
       </c>
       <c r="J99" s="12" t="n">
-        <v>-56.8</v>
+        <v>-915.85</v>
       </c>
       <c r="K99" s="12">
         <f>I99-J99</f>
@@ -6337,9 +6359,11 @@
         <f>IF(K99=0,"",J99/K99)</f>
         <v/>
       </c>
-      <c r="N99" s="10" t="n"/>
+      <c r="N99" s="10" t="n">
+        <v>6.7</v>
+      </c>
       <c r="O99" s="11" t="n">
-        <v>0.79</v>
+        <v>14.91</v>
       </c>
     </row>
     <row r="100">
@@ -6353,12 +6377,12 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
@@ -6367,20 +6391,20 @@
         </is>
       </c>
       <c r="F100" s="4" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="H100" s="4">
         <f>IF(F100*G100=0,"",ROUND(I100/(F100*G100),0))</f>
         <v/>
       </c>
       <c r="I100" s="6" t="n">
-        <v>406</v>
+        <v>108</v>
       </c>
       <c r="J100" s="6" t="n">
-        <v>-1689.42</v>
+        <v>-93.37</v>
       </c>
       <c r="K100" s="6">
         <f>I100-J100</f>
@@ -6394,9 +6418,11 @@
         <f>IF(K100=0,"",J100/K100)</f>
         <v/>
       </c>
-      <c r="N100" s="4" t="n"/>
+      <c r="N100" s="4" t="n">
+        <v>7.5</v>
+      </c>
       <c r="O100" s="5" t="n">
-        <v>7.23</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="101">
@@ -6410,12 +6436,12 @@
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
@@ -6424,20 +6450,20 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G101" s="11" t="n">
-        <v>0.18</v>
+        <v>1.69</v>
       </c>
       <c r="H101" s="10">
         <f>IF(F101*G101=0,"",ROUND(I101/(F101*G101),0))</f>
         <v/>
       </c>
       <c r="I101" s="12" t="n">
-        <v>1080</v>
+        <v>6760</v>
       </c>
       <c r="J101" s="12" t="n">
-        <v>-568.15</v>
+        <v>4974.8</v>
       </c>
       <c r="K101" s="12">
         <f>I101-J101</f>
@@ -6452,10 +6478,10 @@
         <v/>
       </c>
       <c r="N101" s="10" t="n">
-        <v>10.4</v>
+        <v>1302.3</v>
       </c>
       <c r="O101" s="11" t="n">
-        <v>11.4</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="102">
@@ -6469,12 +6495,12 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
@@ -6483,20 +6509,20 @@
         </is>
       </c>
       <c r="F102" s="4" t="n">
-        <v>59</v>
+        <v>120</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="H102" s="4">
         <f>IF(F102*G102=0,"",ROUND(I102/(F102*G102),0))</f>
         <v/>
       </c>
       <c r="I102" s="6" t="n">
-        <v>1062</v>
+        <v>600</v>
       </c>
       <c r="J102" s="6" t="n">
-        <v>-915.85</v>
+        <v>-1741.02</v>
       </c>
       <c r="K102" s="6">
         <f>I102-J102</f>
@@ -6511,10 +6537,10 @@
         <v/>
       </c>
       <c r="N102" s="4" t="n">
-        <v>6.7</v>
+        <v>728</v>
       </c>
       <c r="O102" s="5" t="n">
-        <v>14.91</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="103">
@@ -6528,12 +6554,12 @@
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
@@ -6542,20 +6568,20 @@
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G103" s="11" t="n">
-        <v>0.18</v>
+        <v>1.34</v>
       </c>
       <c r="H103" s="10">
         <f>IF(F103*G103=0,"",ROUND(I103/(F103*G103),0))</f>
         <v/>
       </c>
       <c r="I103" s="12" t="n">
-        <v>108</v>
+        <v>2010</v>
       </c>
       <c r="J103" s="12" t="n">
-        <v>-93.37</v>
+        <v>1653.13</v>
       </c>
       <c r="K103" s="12">
         <f>I103-J103</f>
@@ -6570,10 +6596,10 @@
         <v/>
       </c>
       <c r="N103" s="10" t="n">
-        <v>7.5</v>
+        <v>166.7</v>
       </c>
       <c r="O103" s="11" t="n">
-        <v>1.75</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="104">
@@ -6587,12 +6613,12 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>22:16</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
@@ -6601,20 +6627,20 @@
         </is>
       </c>
       <c r="F104" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G104" s="5" t="n">
-        <v>1.69</v>
+        <v>0</v>
       </c>
       <c r="H104" s="4">
         <f>IF(F104*G104=0,"",ROUND(I104/(F104*G104),0))</f>
         <v/>
       </c>
       <c r="I104" s="6" t="n">
-        <v>6760</v>
+        <v>0</v>
       </c>
       <c r="J104" s="6" t="n">
-        <v>4974.8</v>
+        <v>-2160</v>
       </c>
       <c r="K104" s="6">
         <f>I104-J104</f>
@@ -6629,10 +6655,10 @@
         <v/>
       </c>
       <c r="N104" s="4" t="n">
-        <v>1302.3</v>
+        <v>1854.7</v>
       </c>
       <c r="O104" s="5" t="n">
-        <v>11.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -6646,12 +6672,12 @@
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>22:16</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
@@ -6660,20 +6686,20 @@
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="G105" s="11" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H105" s="10">
         <f>IF(F105*G105=0,"",ROUND(I105/(F105*G105),0))</f>
         <v/>
       </c>
       <c r="I105" s="12" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="J105" s="12" t="n">
-        <v>-1741.02</v>
+        <v>-2500</v>
       </c>
       <c r="K105" s="12">
         <f>I105-J105</f>
@@ -6688,243 +6714,66 @@
         <v/>
       </c>
       <c r="N105" s="10" t="n">
-        <v>728</v>
+        <v>2083.2</v>
       </c>
       <c r="O105" s="11" t="n">
-        <v>37.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>שישי</t>
-        </is>
-      </c>
-      <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>12:54</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="E106" s="3" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
-      <c r="F106" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G106" s="5" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="H106" s="4">
-        <f>IF(F106*G106=0,"",ROUND(I106/(F106*G106),0))</f>
-        <v/>
-      </c>
-      <c r="I106" s="6" t="n">
-        <v>2010</v>
-      </c>
-      <c r="J106" s="6" t="n">
-        <v>1653.13</v>
-      </c>
-      <c r="K106" s="6">
-        <f>I106-J106</f>
-        <v/>
-      </c>
-      <c r="L106" s="5">
-        <f>IF(OR(F106=0,H106=""),"",K106/(F106*H106))</f>
-        <v/>
-      </c>
-      <c r="M106" s="7">
+      <c r="E106" s="14" t="inlineStr">
+        <is>
+          <t>סה"כ</t>
+        </is>
+      </c>
+      <c r="F106" s="15">
+        <f>SUM(F2:F105)</f>
+        <v/>
+      </c>
+      <c r="I106" s="16">
+        <f>SUM(I2:I105)</f>
+        <v/>
+      </c>
+      <c r="J106" s="16">
+        <f>SUM(J2:J105)</f>
+        <v/>
+      </c>
+      <c r="K106" s="16">
+        <f>SUM(K2:K105)</f>
+        <v/>
+      </c>
+      <c r="M106" s="17">
         <f>IF(K106=0,"",J106/K106)</f>
         <v/>
       </c>
-      <c r="N106" s="4" t="n">
-        <v>166.7</v>
-      </c>
-      <c r="O106" s="5" t="n">
-        <v>4.1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B107" s="9" t="inlineStr">
-        <is>
-          <t>שישי</t>
-        </is>
-      </c>
-      <c r="C107" s="9" t="inlineStr">
-        <is>
-          <t>22:16</t>
-        </is>
-      </c>
-      <c r="D107" s="9" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="E107" s="9" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
-      <c r="F107" s="10" t="n">
-        <v>60</v>
-      </c>
-      <c r="G107" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H107" s="10">
-        <f>IF(F107*G107=0,"",ROUND(I107/(F107*G107),0))</f>
-        <v/>
-      </c>
-      <c r="I107" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J107" s="12" t="n">
-        <v>-2160</v>
-      </c>
-      <c r="K107" s="12">
-        <f>I107-J107</f>
-        <v/>
-      </c>
-      <c r="L107" s="11">
-        <f>IF(OR(F107=0,H107=""),"",K107/(F107*H107))</f>
-        <v/>
-      </c>
-      <c r="M107" s="13">
-        <f>IF(K107=0,"",J107/K107)</f>
-        <v/>
-      </c>
-      <c r="N107" s="10" t="n">
-        <v>1854.7</v>
-      </c>
-      <c r="O107" s="11" t="n">
-        <v>0</v>
+      <c r="O106" s="18">
+        <f>SUM(O2:O105)</f>
+        <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>שישי</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>22:16</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>PURR</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
-      <c r="F108" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="G108" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" s="4">
-        <f>IF(F108*G108=0,"",ROUND(I108/(F108*G108),0))</f>
-        <v/>
-      </c>
-      <c r="I108" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" s="6" t="n">
-        <v>-2500</v>
-      </c>
-      <c r="K108" s="6">
-        <f>I108-J108</f>
-        <v/>
-      </c>
-      <c r="L108" s="5">
-        <f>IF(OR(F108=0,H108=""),"",K108/(F108*H108))</f>
-        <v/>
-      </c>
-      <c r="M108" s="7">
-        <f>IF(K108=0,"",J108/K108)</f>
-        <v/>
-      </c>
-      <c r="N108" s="4" t="n">
-        <v>2083.2</v>
-      </c>
-      <c r="O108" s="5" t="n">
-        <v>0</v>
+      <c r="A108" s="19" t="inlineStr">
+        <is>
+          <t>פרמיה ששולמה = תמורה פחות תוצאה נטו. מחיר כניסה = פרמיה / (כמות × מכפיל).</t>
+        </is>
       </c>
     </row>
     <row r="109">
-      <c r="E109" s="14" t="inlineStr">
-        <is>
-          <t>סה"כ</t>
-        </is>
-      </c>
-      <c r="F109" s="15">
-        <f>SUM(F2:F108)</f>
-        <v/>
-      </c>
-      <c r="I109" s="16">
-        <f>SUM(I2:I108)</f>
-        <v/>
-      </c>
-      <c r="J109" s="16">
-        <f>SUM(J2:J108)</f>
-        <v/>
-      </c>
-      <c r="K109" s="16">
-        <f>SUM(K2:K108)</f>
-        <v/>
-      </c>
-      <c r="M109" s="17">
-        <f>IF(K109=0,"",J109/K109)</f>
-        <v/>
-      </c>
-      <c r="O109" s="18">
-        <f>SUM(O2:O108)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="19" t="inlineStr">
-        <is>
-          <t>פרמיה ששולמה = תמורה פחות תוצאה נטו. מחיר כניסה = פרמיה / (כמות × מכפיל).</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="19" t="inlineStr">
+      <c r="A109" s="19" t="inlineStr">
         <is>
           <t>התוצאה נטו כפי שמדווחת ב-IBKR כבר מנוכה עמלות משתי רגלי הסיבוב.</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="19" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="19" t="inlineStr">
         <is>
           <t>מקור: Interactive Brokers, get_account_trades. שעות בשעון המסחר.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O108"/>
+  <autoFilter ref="A1:O105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6991,23 +6840,23 @@
         </is>
       </c>
       <c r="B2" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A2)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A2)</f>
         <v/>
       </c>
       <c r="C2" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A2,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A2,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D2" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A2,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A2,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E2" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A2,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A2,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F2" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A2,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A2,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G2" s="24">
@@ -7022,23 +6871,23 @@
         </is>
       </c>
       <c r="B3" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A3)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A3)</f>
         <v/>
       </c>
       <c r="C3" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A3,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A3,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D3" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A3,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A3,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E3" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A3,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A3,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F3" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A3,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A3,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G3" s="28">
@@ -7053,23 +6902,23 @@
         </is>
       </c>
       <c r="B4" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A4)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A4,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A4,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D4" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A4,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A4,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E4" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A4,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A4,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F4" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A4,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A4,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G4" s="24">
@@ -7080,27 +6929,27 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>NU</t>
         </is>
       </c>
       <c r="B5" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A5)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A5,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A5,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D5" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A5,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A5,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E5" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A5,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A5,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F5" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A5,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A5,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G5" s="28">
@@ -7111,27 +6960,27 @@
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>AAOI</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B6" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A6)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A6,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A6,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D6" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A6,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A6,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E6" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A6,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A6,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F6" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A6,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A6,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G6" s="24">
@@ -7142,27 +6991,27 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>AAOI</t>
         </is>
       </c>
       <c r="B7" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A7)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A7,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A7,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D7" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A7,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A7,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E7" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A7,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A7,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F7" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A7,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A7,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G7" s="28">
@@ -7173,27 +7022,27 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B8" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A8)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A8,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A8,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D8" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A8,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A8,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E8" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A8,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A8,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F8" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A8,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A8,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G8" s="24">
@@ -7204,27 +7053,27 @@
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B9" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A9)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A9,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A9,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D9" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A9,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A9,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E9" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A9,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A9,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F9" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A9,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A9,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G9" s="28">
@@ -7235,27 +7084,27 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B10" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A10)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A10,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A10,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A10,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A10,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E10" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A10,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A10,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F10" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A10,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A10,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G10" s="24">
@@ -7266,27 +7115,27 @@
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B11" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A11)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A11,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A11,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D11" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A11,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A11,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A11,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A11,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A11,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A11,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -7297,27 +7146,27 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B12" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A12)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A12,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A12,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A12,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A12,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E12" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A12,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A12,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F12" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A12,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A12,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G12" s="24">
@@ -7328,27 +7177,27 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A13)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A13,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A13,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D13" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A13,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A13,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E13" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A13,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A13,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F13" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A13,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A13,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G13" s="28">
@@ -7359,27 +7208,27 @@
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B14" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A14)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A14,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A14,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D14" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A14,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A14,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E14" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A14,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A14,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F14" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A14,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A14,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G14" s="24">
@@ -7390,27 +7239,27 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>OKLO</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A15)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A15,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A15,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D15" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A15,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A15,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E15" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A15,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A15,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F15" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A15,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A15,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G15" s="28">
@@ -7421,27 +7270,27 @@
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>OKLO</t>
         </is>
       </c>
       <c r="B16" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A16)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A16,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A16,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D16" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A16,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A16,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E16" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A16,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A16,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F16" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A16,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A16,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G16" s="24">
@@ -7452,27 +7301,27 @@
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A17)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A17,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A17,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D17" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A17,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A17,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E17" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A17,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A17,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F17" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A17,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A17,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G17" s="28">
@@ -7483,27 +7332,27 @@
     <row r="18">
       <c r="A18" s="21" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="B18" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A18)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A18,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A18,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D18" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A18,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A18,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E18" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A18,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A18,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F18" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A18,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A18,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G18" s="24">
@@ -7514,27 +7363,27 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>NU</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A19)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A19,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A19,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D19" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A19,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A19,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E19" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A19,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A19,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F19" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A19,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A19,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G19" s="28">
@@ -7549,23 +7398,23 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A20)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A20,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A20,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D20" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A20,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A20,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E20" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A20,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A20,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F20" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A20,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A20,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G20" s="24">
@@ -7580,23 +7429,23 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A21)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A21,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A21,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D21" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A21,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A21,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E21" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A21,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A21,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F21" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A21,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A21,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G21" s="28">
@@ -7611,23 +7460,23 @@
         </is>
       </c>
       <c r="B22" s="22">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A22)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="22">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A22,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A22,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A22,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A22,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E22" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A22,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A22,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F22" s="23">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A22,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A22,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G22" s="24">
@@ -7642,23 +7491,23 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIF(עסקאות!$D$2:$D$108,$A23)</f>
+        <f>COUNTIF(עסקאות!$D$2:$D$105,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="26">
-        <f>COUNTIFS(עסקאות!$D$2:$D$108,$A23,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$D$2:$D$105,$A23,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="D23" s="26">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A23,עסקאות!$F$2:$F$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A23,עסקאות!$F$2:$F$105)</f>
         <v/>
       </c>
       <c r="E23" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A23,עסקאות!$K$2:$K$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A23,עסקאות!$K$2:$K$105)</f>
         <v/>
       </c>
       <c r="F23" s="27">
-        <f>SUMIF(עסקאות!$D$2:$D$108,$A23,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$D$2:$D$105,$A23,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="G23" s="28">
@@ -7768,15 +7617,15 @@
         </is>
       </c>
       <c r="C2" s="22">
-        <f>COUNTIF(עסקאות!$A$2:$A$108,$A2)</f>
+        <f>COUNTIF(עסקאות!$A$2:$A$105,$A2)</f>
         <v/>
       </c>
       <c r="D2" s="22">
-        <f>COUNTIFS(עסקאות!$A$2:$A$108,$A2,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$A$2:$A$105,$A2,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="E2" s="23">
-        <f>SUMIF(עסקאות!$A$2:$A$108,$A2,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$A$2:$A$105,$A2,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="F2" s="23">
@@ -7794,15 +7643,15 @@
         </is>
       </c>
       <c r="C3" s="22">
-        <f>COUNTIF(עסקאות!$A$2:$A$108,$A3)</f>
+        <f>COUNTIF(עסקאות!$A$2:$A$105,$A3)</f>
         <v/>
       </c>
       <c r="D3" s="22">
-        <f>COUNTIFS(עסקאות!$A$2:$A$108,$A3,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$A$2:$A$105,$A3,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="E3" s="23">
-        <f>SUMIF(עסקאות!$A$2:$A$108,$A3,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$A$2:$A$105,$A3,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="F3" s="23">
@@ -7820,15 +7669,15 @@
         </is>
       </c>
       <c r="C4" s="22">
-        <f>COUNTIF(עסקאות!$A$2:$A$108,$A4)</f>
+        <f>COUNTIF(עסקאות!$A$2:$A$105,$A4)</f>
         <v/>
       </c>
       <c r="D4" s="22">
-        <f>COUNTIFS(עסקאות!$A$2:$A$108,$A4,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$A$2:$A$105,$A4,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="E4" s="23">
-        <f>SUMIF(עסקאות!$A$2:$A$108,$A4,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$A$2:$A$105,$A4,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="F4" s="23">
@@ -7846,15 +7695,15 @@
         </is>
       </c>
       <c r="C5" s="22">
-        <f>COUNTIF(עסקאות!$A$2:$A$108,$A5)</f>
+        <f>COUNTIF(עסקאות!$A$2:$A$105,$A5)</f>
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>COUNTIFS(עסקאות!$A$2:$A$108,$A5,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$A$2:$A$105,$A5,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="E5" s="23">
-        <f>SUMIF(עסקאות!$A$2:$A$108,$A5,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$A$2:$A$105,$A5,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="F5" s="23">
@@ -7872,15 +7721,15 @@
         </is>
       </c>
       <c r="C6" s="22">
-        <f>COUNTIF(עסקאות!$A$2:$A$108,$A6)</f>
+        <f>COUNTIF(עסקאות!$A$2:$A$105,$A6)</f>
         <v/>
       </c>
       <c r="D6" s="22">
-        <f>COUNTIFS(עסקאות!$A$2:$A$108,$A6,עסקאות!$J$2:$J$108,"&gt;0")</f>
+        <f>COUNTIFS(עסקאות!$A$2:$A$105,$A6,עסקאות!$J$2:$J$105,"&gt;0")</f>
         <v/>
       </c>
       <c r="E6" s="23">
-        <f>SUMIF(עסקאות!$A$2:$A$108,$A6,עסקאות!$J$2:$J$108)</f>
+        <f>SUMIF(עסקאות!$A$2:$A$105,$A6,עסקאות!$J$2:$J$105)</f>
         <v/>
       </c>
       <c r="F6" s="23">
@@ -7918,7 +7767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -7972,11 +7821,11 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>(-) מכירות ב-0 ללא פוזיציה פתוחה — שאריות ריסטרט</t>
+          <t>(-) פוזיציות שנעלמו בריסט של חשבון הדמה (CRM, NU, NVDA)</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="C4" s="23" t="n">
         <v>0</v>
@@ -7985,77 +7834,90 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>(=) שורות פקיעה — נזקפות כהפסד מלא</t>
+          <t>(-) מכירות ב-0 ללא פוזיציה פתוחה — שאריות ריסטרט</t>
         </is>
       </c>
       <c r="B5" s="26" t="n">
-        <v>5</v>
+        <v>-3</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>-11171</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>(-) רגלי BUY</t>
+          <t>(=) שורות פקיעה — נזקפות כהפסד מלא</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>-335</v>
+        <v>2</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>5064.34</v>
+        <v>-4660</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>(-) טיקרים שאינם ברשימה שנמסרה</t>
+          <t>(-) רגלי BUY</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>-46</v>
+        <v>-335</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>11606.97</v>
+        <v>5064.34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
+          <t>(-) טיקרים שאינם ברשימה שנמסרה</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>-46</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>11606.97</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
           <t>(-) פוזיציות שהועברו ללילה (ANET, MRNA)</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B9" s="26" t="n">
         <v>-9</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C9" s="27" t="n">
         <v>2519.7</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="14">
+    <row r="10">
+      <c r="A10" s="14">
         <f> הסט המסונן (גיליון "עסקאות")</f>
         <v/>
       </c>
-      <c r="B9" s="15">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="16">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="B10" s="15">
+        <f>SUM(B2:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="16">
+        <f>SUM(C2:C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>בדיקת התאמה מול גיליון העסקאות</t>
         </is>
       </c>
-      <c r="C10" s="31">
-        <f>'עסקאות'!J109</f>
+      <c r="C11" s="31">
+        <f>'עסקאות'!J106</f>
         <v/>
       </c>
     </row>

</xml_diff>